<commit_message>
Tighten natal whole-passage review
</commit_message>
<xml_diff>
--- a/packages/astro-knowledge/review/TLDR-LL-V13-WP1-BATCH-01-EDITORIAL-REVISION-V3.xlsx
+++ b/packages/astro-knowledge/review/TLDR-LL-V13-WP1-BATCH-01-EDITORIAL-REVISION-V3.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R053de5d1a6c14e7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchSummary" sheetId="2" r:id="Rb0650d67d5e64137"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates132" sheetId="3" r:id="R876216ff6b684294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V3 Method" sheetId="4" r:id="R0222ee6d3fb7469f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1f5c67926efb4443"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchSummary" sheetId="2" r:id="Rfa90a6703d4b4943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates132" sheetId="3" r:id="R5045d0a609ae4cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V3 Method" sheetId="4" r:id="R642aa2e09d064bc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -48,7 +48,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -122,6 +122,11 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD9E2F3"/>
       </x:patternFill>
     </x:fill>
@@ -166,7 +171,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="87">
+  <x:cellXfs count="90">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -350,20 +355,27 @@
     <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1158,6 +1170,9 @@
     <x:col min="19" max="19" width="32" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="58" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="34" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="28" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1246,13 +1261,22 @@
         <x:v>Fresh copy (V3 mechanism method, NOT owner approved)</x:v>
       </x:c>
       <x:c r="S1" s="66" t="str">
-        <x:v>V3 deterministic gate</x:v>
+        <x:v>V3 deterministic precheck (NOT an editorial verdict)</x:v>
       </x:c>
       <x:c r="T1" s="66" t="str">
         <x:v>V3 owner verdict</x:v>
       </x:c>
       <x:c r="U1" s="66" t="str">
         <x:v>V3 owner edit</x:v>
+      </x:c>
+      <x:c r="V1" s="66" t="str">
+        <x:v>Photograph-test minimum</x:v>
+      </x:c>
+      <x:c r="W1" s="66" t="str">
+        <x:v>Whole-passage semantic review</x:v>
+      </x:c>
+      <x:c r="X1" s="66" t="str">
+        <x:v>Row-by-row comparison note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1327,6 +1351,13 @@
       </x:c>
       <x:c r="T2" s="78"/>
       <x:c r="U2" s="78"/>
+      <x:c r="V2" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W2" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X2" s="78"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="41" t="n">
@@ -1400,6 +1431,13 @@
       </x:c>
       <x:c r="T3" s="78"/>
       <x:c r="U3" s="78"/>
+      <x:c r="V3" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W3" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X3" s="78"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="40" t="n">
@@ -1471,10 +1509,17 @@
         <x:v>You keep the plan alive when everybody else is ready to cancel it. A difficult week still gets a dinner on the calendar, a stalled project gets another try, and a disappointed friend hears a reason the story may not be over. The same hope can keep you paying for a promise after the receipts say it is not working. Optimism helps most when it can look at the facts without replacing them.</x:v>
       </x:c>
       <x:c r="S4" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T4" s="78"/>
       <x:c r="U4" s="78"/>
+      <x:c r="V4" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W4" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X4" s="78"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="41" t="n">
@@ -1546,10 +1591,17 @@
         <x:v>People start looking at you when the meeting reaches the decision nobody wants to make. You can name the larger stakes, gather support, and move a group toward a bolder plan. The temptation is to treat every objection as a delay you are entitled to remove. Influence becomes easier to trust when disagreement is allowed to change the decision.</x:v>
       </x:c>
       <x:c r="S5" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T5" s="78"/>
       <x:c r="U5" s="78"/>
+      <x:c r="V5" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W5" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X5" s="78"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="40" t="n">
@@ -1621,10 +1673,17 @@
         <x:v>The larger plan feels possible once the budget, deadline, and next three steps are on the page. You can take an ambitious idea and give it enough structure to survive the first difficult month. That same need for a sound plan can keep you revising the spreadsheet after the work is ready to begin. Expansion and caution share one desk here, and neither one gets to make every decision.</x:v>
       </x:c>
       <x:c r="S6" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T6" s="78"/>
       <x:c r="U6" s="78"/>
+      <x:c r="V6" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W6" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X6" s="78"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="41" t="n">
@@ -1698,6 +1757,13 @@
       </x:c>
       <x:c r="T7" s="78"/>
       <x:c r="U7" s="78"/>
+      <x:c r="V7" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W7" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X7" s="78"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="40" t="n">
@@ -1771,6 +1837,13 @@
       </x:c>
       <x:c r="T8" s="78"/>
       <x:c r="U8" s="78"/>
+      <x:c r="V8" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W8" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X8" s="78"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="41" t="n">
@@ -1842,10 +1915,17 @@
         <x:v>An unfinished project can make the whole week feel like evidence that you are falling behind. You start over, change the plan, or hide the draft because the current version does not yet deserve your name. The standard across the room keeps moving just as the work approaches it. Finishing becomes possible when a rough version is allowed to exist long enough to be improved.</x:v>
       </x:c>
       <x:c r="S9" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T9" s="78"/>
       <x:c r="U9" s="78"/>
+      <x:c r="V9" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W9" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X9" s="78"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="40" t="n">
@@ -1919,6 +1999,13 @@
       </x:c>
       <x:c r="T10" s="78"/>
       <x:c r="U10" s="78"/>
+      <x:c r="V10" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W10" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X10" s="78"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="41" t="n">
@@ -1990,10 +2077,17 @@
         <x:v>A conversation about one belief can become a referendum on everybody else's freedom. You defend the position that helped you leave an old rule, then get impatient when another person uses the same independence to choose differently. The argument grows because conviction is standing across from somebody else's right to change the terms. A view does not become weaker because another person remains unconvinced.</x:v>
       </x:c>
       <x:c r="S11" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T11" s="78"/>
       <x:c r="U11" s="78"/>
+      <x:c r="V11" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W11" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X11" s="78"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="n">
@@ -2067,6 +2161,13 @@
       </x:c>
       <x:c r="T12" s="78"/>
       <x:c r="U12" s="78"/>
+      <x:c r="V12" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W12" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X12" s="78"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="41" t="n">
@@ -2140,6 +2241,13 @@
       </x:c>
       <x:c r="T13" s="78"/>
       <x:c r="U13" s="78"/>
+      <x:c r="V13" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W13" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X13" s="78"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="n">
@@ -2213,6 +2321,13 @@
       </x:c>
       <x:c r="T14" s="78"/>
       <x:c r="U14" s="78"/>
+      <x:c r="V14" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W14" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X14" s="78"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="41" t="n">
@@ -2286,6 +2401,13 @@
       </x:c>
       <x:c r="T15" s="78"/>
       <x:c r="U15" s="78"/>
+      <x:c r="V15" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W15" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X15" s="78"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="40" t="n">
@@ -2359,6 +2481,13 @@
       </x:c>
       <x:c r="T16" s="78"/>
       <x:c r="U16" s="78"/>
+      <x:c r="V16" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W16" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X16" s="78"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="41" t="n">
@@ -2430,10 +2559,17 @@
         <x:v>You can walk into a complicated meeting, find the decision underneath the speeches, and help the group deal with it. Large changes feel less frightening when you can see how the system, the people, and the consequences fit together. That ease can put more influence in your hands before anyone formally names it. The useful part is not having the last word; it is knowing which change will still hold after the room empties.</x:v>
       </x:c>
       <x:c r="S17" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T17" s="78"/>
       <x:c r="U17" s="78"/>
+      <x:c r="V17" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W17" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X17" s="78"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="40" t="n">
@@ -2507,6 +2643,13 @@
       </x:c>
       <x:c r="T18" s="78"/>
       <x:c r="U18" s="78"/>
+      <x:c r="V18" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W18" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X18" s="78"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="41" t="n">
@@ -2578,10 +2721,17 @@
         <x:v>A strange idea gets your attention before its unfamiliarity becomes a reason to dismiss it. You read the article, ask the unexpected person, or change the route because the new option makes more sense than the familiar one. Curiosity and judgment cooperate well enough that a different view can improve the plan without overturning your whole life. People often remember that you made room for an idea before it was popular.</x:v>
       </x:c>
       <x:c r="S19" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T19" s="78"/>
       <x:c r="U19" s="78"/>
+      <x:c r="V19" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W19" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X19" s="78"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="40" t="n">
@@ -2655,6 +2805,13 @@
       </x:c>
       <x:c r="T20" s="78"/>
       <x:c r="U20" s="78"/>
+      <x:c r="V20" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W20" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X20" s="78"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="41" t="n">
@@ -2728,6 +2885,13 @@
       </x:c>
       <x:c r="T21" s="78"/>
       <x:c r="U21" s="78"/>
+      <x:c r="V21" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W21" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X21" s="78"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="40" t="n">
@@ -2799,10 +2963,17 @@
         <x:v>You can work for hours when the purpose feels vivid, then stare at the same task when that feeling disappears. Effort follows the picture in your head, so a project with meaning gets your whole body while an ordinary deadline can be strangely hard to start. This makes inspiration powerful and consistency uneven. The work becomes more dependable when the next action is written down before the mood changes.</x:v>
       </x:c>
       <x:c r="S22" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T22" s="78"/>
       <x:c r="U22" s="78"/>
+      <x:c r="V22" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W22" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X22" s="78"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="41" t="n">
@@ -2876,6 +3047,13 @@
       </x:c>
       <x:c r="T23" s="78"/>
       <x:c r="U23" s="78"/>
+      <x:c r="V23" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W23" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X23" s="78"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="40" t="n">
@@ -2947,10 +3125,17 @@
         <x:v>Once you decide the heavy desk has to move, the difficult call has to happen, or the stalled project has to finish, very little distracts you. Pressure tends to concentrate your effort instead of scattering it. That force can carry a group through a hard job, and it can also make another person's hesitation feel like interference. Determination works differently from control, even when both get the room moving.</x:v>
       </x:c>
       <x:c r="S24" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T24" s="78"/>
       <x:c r="U24" s="78"/>
+      <x:c r="V24" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W24" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X24" s="78"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="41" t="n">
@@ -3024,6 +3209,13 @@
       </x:c>
       <x:c r="T25" s="78"/>
       <x:c r="U25" s="78"/>
+      <x:c r="V25" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W25" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X25" s="78"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="40" t="n">
@@ -3097,6 +3289,13 @@
       </x:c>
       <x:c r="T26" s="78"/>
       <x:c r="U26" s="78"/>
+      <x:c r="V26" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W26" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X26" s="78"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="41" t="n">
@@ -3170,6 +3369,13 @@
       </x:c>
       <x:c r="T27" s="78"/>
       <x:c r="U27" s="78"/>
+      <x:c r="V27" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W27" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X27" s="78"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="40" t="n">
@@ -3241,10 +3447,17 @@
         <x:v>A confident answer can come out before you have checked the document behind it. When you already feel outmatched, taking credit, enlarging the story, or promising more than you can deliver offers a quick way to feel capable. The relief lasts until another person asks for the file, date, or result. Action gets cleaner when the proof can stand across from the claim.</x:v>
       </x:c>
       <x:c r="S28" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T28" s="78"/>
       <x:c r="U28" s="78"/>
+      <x:c r="V28" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W28" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X28" s="78"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="41" t="n">
@@ -3318,6 +3531,13 @@
       </x:c>
       <x:c r="T29" s="78"/>
       <x:c r="U29" s="78"/>
+      <x:c r="V29" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W29" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X29" s="78"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="40" t="n">
@@ -3391,6 +3611,13 @@
       </x:c>
       <x:c r="T30" s="78"/>
       <x:c r="U30" s="78"/>
+      <x:c r="V30" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W30" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X30" s="78"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="41" t="n">
@@ -3464,6 +3691,13 @@
       </x:c>
       <x:c r="T31" s="78"/>
       <x:c r="U31" s="78"/>
+      <x:c r="V31" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W31" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X31" s="78"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="40" t="n">
@@ -3537,6 +3771,13 @@
       </x:c>
       <x:c r="T32" s="78"/>
       <x:c r="U32" s="78"/>
+      <x:c r="V32" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W32" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X32" s="78"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="41" t="n">
@@ -3608,10 +3849,17 @@
         <x:v>A missed workout, rejected proposal, or unfinished task can land like a verdict on your worth. You push harder to erase the feeling, then lose momentum when effort does not produce an immediate result. The square turns one setback into a fight between action and doubt. A failed project is information about the attempt; it is not a biography.</x:v>
       </x:c>
       <x:c r="S33" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T33" s="78"/>
       <x:c r="U33" s="78"/>
+      <x:c r="V33" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W33" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X33" s="78"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="40" t="n">
@@ -3685,6 +3933,13 @@
       </x:c>
       <x:c r="T34" s="78"/>
       <x:c r="U34" s="78"/>
+      <x:c r="V34" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W34" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X34" s="78"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="41" t="n">
@@ -3758,6 +4013,13 @@
       </x:c>
       <x:c r="T35" s="78"/>
       <x:c r="U35" s="78"/>
+      <x:c r="V35" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W35" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X35" s="78"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="40" t="n">
@@ -3831,6 +4093,13 @@
       </x:c>
       <x:c r="T36" s="78"/>
       <x:c r="U36" s="78"/>
+      <x:c r="V36" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W36" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X36" s="78"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="41" t="n">
@@ -3904,6 +4173,13 @@
       </x:c>
       <x:c r="T37" s="78"/>
       <x:c r="U37" s="78"/>
+      <x:c r="V37" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W37" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X37" s="78"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="40" t="n">
@@ -3975,10 +4251,17 @@
         <x:v>You can stay with the difficult job after the room gets tired of talking about it. A heavy move, long repair, or tense negotiation brings out steady force rather than panic. You tend to know when to push, when to wait, and where one decisive action will matter most. People may experience that control as calm because they see the result before they see the effort behind it.</x:v>
       </x:c>
       <x:c r="S38" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T38" s="78"/>
       <x:c r="U38" s="78"/>
+      <x:c r="V38" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W38" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X38" s="78"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="41" t="n">
@@ -4052,6 +4335,13 @@
       </x:c>
       <x:c r="T39" s="78"/>
       <x:c r="U39" s="78"/>
+      <x:c r="V39" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W39" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X39" s="78"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="40" t="n">
@@ -4125,6 +4415,13 @@
       </x:c>
       <x:c r="T40" s="78"/>
       <x:c r="U40" s="78"/>
+      <x:c r="V40" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W40" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X40" s="78"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="41" t="n">
@@ -4196,10 +4493,17 @@
         <x:v>The answer is often out of your mouth while somebody else is still building the question. You spot the weak point, name it quickly, and can turn a slow meeting into an actual decision. The same speed gives words an edge, especially when waiting feels like losing the argument. A fast mind can still leave enough room for the other sentence to finish.</x:v>
       </x:c>
       <x:c r="S41" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T41" s="78"/>
       <x:c r="U41" s="78"/>
+      <x:c r="V41" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W41" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X41" s="78"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="40" t="n">
@@ -4273,6 +4577,13 @@
       </x:c>
       <x:c r="T42" s="78"/>
       <x:c r="U42" s="78"/>
+      <x:c r="V42" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W42" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X42" s="78"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="41" t="n">
@@ -4344,10 +4655,17 @@
         <x:v>You notice the pause in a phone call, the mood in an email, or the image that makes an idea finally click. Meaning often arrives through tone and association before it arrives as a clean list of facts. That sensitivity can make writing, music, and conversation unusually vivid. It can also make an impression feel documented before the document has been checked.</x:v>
       </x:c>
       <x:c r="S43" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T43" s="78"/>
       <x:c r="U43" s="78"/>
+      <x:c r="V43" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W43" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X43" s="78"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="40" t="n">
@@ -4421,6 +4739,13 @@
       </x:c>
       <x:c r="T44" s="78"/>
       <x:c r="U44" s="78"/>
+      <x:c r="V44" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W44" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X44" s="78"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="41" t="n">
@@ -4492,10 +4817,17 @@
         <x:v>A simple answer usually produces the next question. You reread the contract, search the archive, or keep the conversation going until the part nobody named is on the table. This can make you an exacting researcher and a difficult person to distract with a polished explanation. The mind keeps digging here, and it needs to know when the answer underneath the answer has actually been found.</x:v>
       </x:c>
       <x:c r="S45" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T45" s="78"/>
       <x:c r="U45" s="78"/>
+      <x:c r="V45" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W45" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X45" s="78"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="40" t="n">
@@ -4567,10 +4899,17 @@
         <x:v>You can sit with a difficult document until every sentence means what it says. Thought slows down enough to test the claim, organize the evidence, and notice the consequence somebody else skipped. That weight makes your words dependable, but it can also make an ordinary reply feel like something that must be perfect before it is sent. Silence is not always a more accurate answer.</x:v>
       </x:c>
       <x:c r="S46" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T46" s="78"/>
       <x:c r="U46" s="78"/>
+      <x:c r="V46" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W46" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X46" s="78"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="41" t="n">
@@ -4644,6 +4983,13 @@
       </x:c>
       <x:c r="T47" s="78"/>
       <x:c r="U47" s="78"/>
+      <x:c r="V47" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W47" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X47" s="78"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="40" t="n">
@@ -4715,10 +5061,17 @@
         <x:v>You rewrite the tense email once before sending it and find the sentence that lets the point land without humiliating anybody. Language tends to move toward agreement, beauty, or a form people can hear. That helps with editing, design, negotiation, and difficult conversations. The cost appears when keeping the exchange pleasant matters more than saying the part that could change it.</x:v>
       </x:c>
       <x:c r="S48" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T48" s="78"/>
       <x:c r="U48" s="78"/>
+      <x:c r="V48" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W48" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X48" s="78"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="41" t="n">
@@ -4792,6 +5145,13 @@
       </x:c>
       <x:c r="T49" s="78"/>
       <x:c r="U49" s="78"/>
+      <x:c r="V49" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W49" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X49" s="78"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="40" t="n">
@@ -4863,10 +5223,17 @@
         <x:v>The story gets bigger while you are telling it. One example becomes a rule, the headline travels farther than the article, and a generous promise reaches the room before the calendar or budget has been checked. The mind sees the large pattern while the missing detail waits across from it. A persuasive idea still needs the date, number, and source that can hold it up.</x:v>
       </x:c>
       <x:c r="S50" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T50" s="78"/>
       <x:c r="U50" s="78"/>
+      <x:c r="V50" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W50" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X50" s="78"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="41" t="n">
@@ -4938,10 +5305,17 @@
         <x:v>A disagreement can keep running in your head long after the call ends. You draft the reply, rehearse the next point, answer before the other person finishes, and discover that your body has been braced through the whole exchange. Thought and action pull on opposite ends of the conversation. The sharpest response is not always the one that reaches the actual issue.</x:v>
       </x:c>
       <x:c r="S51" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T51" s="78"/>
       <x:c r="U51" s="78"/>
+      <x:c r="V51" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W51" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X51" s="78"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="40" t="n">
@@ -5015,6 +5389,13 @@
       </x:c>
       <x:c r="T52" s="78"/>
       <x:c r="U52" s="78"/>
+      <x:c r="V52" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W52" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X52" s="78"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="41" t="n">
@@ -5086,10 +5467,17 @@
         <x:v>A correction can feel less like new information and more like somebody trying to take the floor away from you. You defend the sentence, question their source, and keep arguing after the original point has disappeared. The opposition makes disagreement carry more power than the topic alone explains. The conversation changes when being wrong about one fact no longer means losing your whole position.</x:v>
       </x:c>
       <x:c r="S53" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T53" s="78"/>
       <x:c r="U53" s="78"/>
+      <x:c r="V53" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W53" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X53" s="78"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="40" t="n">
@@ -5161,10 +5549,17 @@
         <x:v>A short reply can sound like rejection before you have finished reading it. You hear the criticism in the pause, the closed door in the delay, or the final no inside a question that was only cautious. The mind keeps meeting a stricter voice across the table. Checking what was actually said can prevent a difficult conversation from becoming a sentence nobody spoke.</x:v>
       </x:c>
       <x:c r="S54" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T54" s="78"/>
       <x:c r="U54" s="78"/>
+      <x:c r="V54" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W54" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X54" s="78"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="41" t="n">
@@ -5238,6 +5633,13 @@
       </x:c>
       <x:c r="T55" s="78"/>
       <x:c r="U55" s="78"/>
+      <x:c r="V55" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W55" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X55" s="78"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="40" t="n">
@@ -5309,10 +5711,17 @@
         <x:v>You can love the new idea until somebody else presents it first. Then the meeting becomes an argument about their wording, timing, or authority instead of a look at what the idea could change. Original thought matters so much that receiving it from across the table can feel strangely irritating. The useful surprise is still useful when your name was not on the first draft.</x:v>
       </x:c>
       <x:c r="S56" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T56" s="78"/>
       <x:c r="U56" s="78"/>
+      <x:c r="V56" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W56" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X56" s="78"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="41" t="n">
@@ -5386,6 +5795,13 @@
       </x:c>
       <x:c r="T57" s="78"/>
       <x:c r="U57" s="78"/>
+      <x:c r="V57" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W57" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X57" s="78"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="40" t="n">
@@ -5459,6 +5875,13 @@
       </x:c>
       <x:c r="T58" s="78"/>
       <x:c r="U58" s="78"/>
+      <x:c r="V58" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W58" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X58" s="78"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="41" t="n">
@@ -5532,6 +5955,13 @@
       </x:c>
       <x:c r="T59" s="78"/>
       <x:c r="U59" s="78"/>
+      <x:c r="V59" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W59" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X59" s="78"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="40" t="n">
@@ -5603,10 +6033,17 @@
         <x:v>You can spend an hour fixing one paragraph and miss the decision the document was supposed to support. Concentration narrows around the error, the caveat, or the rule that cannot be broken. That precision catches problems other people overlook, but the square can make every detail feel equally urgent. The work needs both the exact sentence and the reason the sentence is there.</x:v>
       </x:c>
       <x:c r="S60" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T60" s="78"/>
       <x:c r="U60" s="78"/>
+      <x:c r="V60" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W60" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X60" s="78"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="41" t="n">
@@ -5680,6 +6117,13 @@
       </x:c>
       <x:c r="T61" s="78"/>
       <x:c r="U61" s="78"/>
+      <x:c r="V61" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W61" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X61" s="78"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="40" t="n">
@@ -5753,6 +6197,13 @@
       </x:c>
       <x:c r="T62" s="78"/>
       <x:c r="U62" s="78"/>
+      <x:c r="V62" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W62" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X62" s="78"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="41" t="n">
@@ -5824,10 +6275,17 @@
         <x:v>You can take a crowded set of notes and find the argument that makes the whole presentation easier to follow. Large ideas and practical organization tend to cooperate, so teaching, planning, and explaining feel less like separate jobs. People often leave the conversation understanding both the point and where to look next. The ease can produce several good plans at once, which still have to fit on one calendar.</x:v>
       </x:c>
       <x:c r="S63" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T63" s="78"/>
       <x:c r="U63" s="78"/>
+      <x:c r="V63" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W63" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X63" s="78"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="40" t="n">
@@ -5901,6 +6359,13 @@
       </x:c>
       <x:c r="T64" s="78"/>
       <x:c r="U64" s="78"/>
+      <x:c r="V64" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W64" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X64" s="78"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="41" t="n">
@@ -5974,6 +6439,13 @@
       </x:c>
       <x:c r="T65" s="78"/>
       <x:c r="U65" s="78"/>
+      <x:c r="V65" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W65" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X65" s="78"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="40" t="n">
@@ -6045,10 +6517,17 @@
         <x:v>A difficult subject can hold your attention until the archive, interview, or technical document finally makes sense. You are comfortable staying with the question after easy explanations stop working. That depth helps you master material other people only skim and notice the fact that changes the conclusion. Research becomes satisfying here because the answer has to survive being examined.</x:v>
       </x:c>
       <x:c r="S66" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T66" s="78"/>
       <x:c r="U66" s="78"/>
+      <x:c r="V66" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W66" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X66" s="78"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="41" t="n">
@@ -6120,10 +6599,17 @@
         <x:v>You can explain a complicated rule in the order another person actually needs to hear it. Notes become a lesson, a scattered project gets a sequence, and pressure often makes your thinking more deliberate instead of less clear. The mind has enough structure to stay with difficult material without turning every pause into failure. People tend to trust the answer because they can see how you reached it.</x:v>
       </x:c>
       <x:c r="S67" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T67" s="78"/>
       <x:c r="U67" s="78"/>
+      <x:c r="V67" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W67" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X67" s="78"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="40" t="n">
@@ -6197,6 +6683,13 @@
       </x:c>
       <x:c r="T68" s="78"/>
       <x:c r="U68" s="78"/>
+      <x:c r="V68" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W68" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X68" s="78"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="41" t="n">
@@ -6268,10 +6761,17 @@
         <x:v>The useful shortcut often appears while everybody else is still following the old instructions. You connect two ideas, find a cleaner tool, or say the strange sentence that makes the room understand the problem differently. Original thought moves easily into language here. The best ideas still become more useful after somebody who did not invent them can follow the steps.</x:v>
       </x:c>
       <x:c r="S69" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T69" s="78"/>
       <x:c r="U69" s="78"/>
+      <x:c r="V69" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W69" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X69" s="78"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="40" t="n">
@@ -6345,6 +6845,13 @@
       </x:c>
       <x:c r="T70" s="78"/>
       <x:c r="U70" s="78"/>
+      <x:c r="V70" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W70" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X70" s="78"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="41" t="n">
@@ -6416,10 +6923,17 @@
         <x:v>You often talk your way into knowing what you feel. A text gets longer as the mood becomes clearer, a conversation changes the memory, or the right word finally explains why the whole day felt off. Thought and feeling share the same microphone. This can make emotional honesty immediate, and it can also make a passing mood sound like a settled conclusion.</x:v>
       </x:c>
       <x:c r="S71" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T71" s="78"/>
       <x:c r="U71" s="78"/>
+      <x:c r="V71" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W71" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X71" s="78"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="40" t="n">
@@ -6493,6 +7007,13 @@
       </x:c>
       <x:c r="T72" s="78"/>
       <x:c r="U72" s="78"/>
+      <x:c r="V72" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W72" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X72" s="78"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="41" t="n">
@@ -6566,6 +7087,13 @@
       </x:c>
       <x:c r="T73" s="78"/>
       <x:c r="U73" s="78"/>
+      <x:c r="V73" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W73" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X73" s="78"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="40" t="n">
@@ -6637,10 +7165,17 @@
         <x:v>A late text, changed plan, or careless comment can open a much larger feeling than the event appears to deserve. Once your reaction starts, it is difficult to keep the old fear, the current person, and the actual problem in separate rooms. Small moments carry unusual emotional weight here. The immediate event still needs its own size, even when it touches something deeper.</x:v>
       </x:c>
       <x:c r="S74" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T74" s="78"/>
       <x:c r="U74" s="78"/>
+      <x:c r="V74" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W74" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X74" s="78"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="41" t="n">
@@ -6712,10 +7247,17 @@
         <x:v>You are often the person who makes the call, handles the bill, and keeps the day moving while everybody else is upset. Responsibility provides something firm to do when vulnerability feels less manageable. People may trust your steadiness and miss how much you keep private. Being useful can hold a difficult moment together without answering the question of who gets to comfort you.</x:v>
       </x:c>
       <x:c r="S75" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T75" s="78"/>
       <x:c r="U75" s="78"/>
+      <x:c r="V75" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W75" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X75" s="78"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="40" t="n">
@@ -6789,6 +7331,13 @@
       </x:c>
       <x:c r="T76" s="78"/>
       <x:c r="U76" s="78"/>
+      <x:c r="V76" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W76" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X76" s="78"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="41" t="n">
@@ -6860,10 +7409,17 @@
         <x:v>Your room can feel fine at breakfast and impossible by lunch. A changed plan, unexpected message, or sudden need for space moves through the body before there is time to prepare an explanation. Emotional life updates quickly here, which makes adaptation fast and predictability difficult. Other people may need the new information before they can follow the change.</x:v>
       </x:c>
       <x:c r="S77" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T77" s="78"/>
       <x:c r="U77" s="78"/>
+      <x:c r="V77" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W77" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X77" s="78"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="40" t="n">
@@ -6935,10 +7491,17 @@
         <x:v>You remember the coffee order, bring the extra chair, and notice when somebody needs the gentler version of the truth. Affection and feeling tend to arrive together, so care is often visible in the way a room, meal, or conversation is arranged. That softness draws people in. It can also make their comfort hard to separate from your own mood.</x:v>
       </x:c>
       <x:c r="S78" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T78" s="78"/>
       <x:c r="U78" s="78"/>
+      <x:c r="V78" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W78" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X78" s="78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="41" t="n">
@@ -7010,10 +7573,17 @@
         <x:v>You say yes to the dinner, the extra project, and the early flight because each one sounds worth the effort on its own. The body sends the bill later, when there has not been a proper meal or an empty evening all week. Feeling and possibility pull from opposite sides of the calendar. Generosity is still generous when one invitation has to remain unanswered.</x:v>
       </x:c>
       <x:c r="S79" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T79" s="78"/>
       <x:c r="U79" s="78"/>
+      <x:c r="V79" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W79" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X79" s="78"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="40" t="n">
@@ -7085,10 +7655,17 @@
         <x:v>A friendly game becomes a rematch, a small correction becomes a challenge, or a quiet evening turns into the moment you decide to prove a point. The body reacts before the feeling has a name, and another person can suddenly seem like the opponent. Emotional need and action face each other across the room. Not every charged moment requires a winner.</x:v>
       </x:c>
       <x:c r="S80" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T80" s="78"/>
       <x:c r="U80" s="78"/>
+      <x:c r="V80" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W80" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X80" s="78"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="41" t="n">
@@ -7160,10 +7737,17 @@
         <x:v>The sentence comes out sharper than the feeling underneath it. You argue about the date, wording, or logic while the hurt that started the conversation waits on the other side. The mind can build a strong case and still miss what the body was trying to say. A precise explanation does not automatically make the original feeling easier to hear.</x:v>
       </x:c>
       <x:c r="S81" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T81" s="78"/>
       <x:c r="U81" s="78"/>
+      <x:c r="V81" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W81" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X81" s="78"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="40" t="n">
@@ -7235,10 +7819,17 @@
         <x:v>When you are already upset, a delayed message can become a whole story before the other person replies. Tone, memory, hope, and fear all start supplying evidence, and it becomes difficult to tell what happened from what the moment felt like. Emotion and imagination face each other here. The facts become easier to sort after the first wave is no longer writing them.</x:v>
       </x:c>
       <x:c r="S82" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T82" s="78"/>
       <x:c r="U82" s="78"/>
+      <x:c r="V82" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W82" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X82" s="78"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="41" t="n">
@@ -7312,6 +7903,13 @@
       </x:c>
       <x:c r="T83" s="78"/>
       <x:c r="U83" s="78"/>
+      <x:c r="V83" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W83" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X83" s="78"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="40" t="n">
@@ -7385,6 +7983,13 @@
       </x:c>
       <x:c r="T84" s="78"/>
       <x:c r="U84" s="78"/>
+      <x:c r="V84" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W84" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X84" s="78"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="41" t="n">
@@ -7456,10 +8061,17 @@
         <x:v>You can want somebody close and then need the room back as soon as they arrive. Plans are made warmly, canceled abruptly, and missed once the space is quiet again. Closeness and freedom pull from opposite sides of the same relationship. The change is easier for another person to live with when it is named before the door closes.</x:v>
       </x:c>
       <x:c r="S85" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T85" s="78"/>
       <x:c r="U85" s="78"/>
+      <x:c r="V85" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W85" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X85" s="78"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="40" t="n">
@@ -7531,10 +8143,17 @@
         <x:v>A quiet reply or missed invitation can make affection feel absent even when nothing has actually ended. You reach for another text, another answer, or a nicer version of yourself to restore the warmth. Emotional need keeps looking across the room for proof from Venus. Care from another person can matter without becoming the only evidence that you are okay.</x:v>
       </x:c>
       <x:c r="S86" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T86" s="78"/>
       <x:c r="U86" s="78"/>
+      <x:c r="V86" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W86" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X86" s="78"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="41" t="n">
@@ -7608,6 +8227,13 @@
       </x:c>
       <x:c r="T87" s="78"/>
       <x:c r="U87" s="78"/>
+      <x:c r="V87" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W87" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X87" s="78"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="40" t="n">
@@ -7679,10 +8305,17 @@
         <x:v>A small embarrassment can turn into your long explanation of why the decision was still right. Pride steps in quickly when a vulnerable feeling is exposed, so the story grows while the original hurt gets harder to see. The square makes confidence and emotion press against each other. The room often softens once the feeling no longer needs a larger argument to defend it.</x:v>
       </x:c>
       <x:c r="S88" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T88" s="78"/>
       <x:c r="U88" s="78"/>
+      <x:c r="V88" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W88" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X88" s="78"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="41" t="n">
@@ -7754,10 +8387,17 @@
         <x:v>You can explain the whole situation clearly and still feel worse when the conversation ends. The facts line up, the timeline makes sense, and the heart refuses to sign the report. Thought and feeling keep interrupting each other's version of what happened. The message becomes more honest when both the reason and the reaction are allowed into the same paragraph.</x:v>
       </x:c>
       <x:c r="S89" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T89" s="78"/>
       <x:c r="U89" s="78"/>
+      <x:c r="V89" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W89" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X89" s="78"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="40" t="n">
@@ -7831,6 +8471,13 @@
       </x:c>
       <x:c r="T90" s="78"/>
       <x:c r="U90" s="78"/>
+      <x:c r="V90" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W90" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X90" s="78"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="41" t="n">
@@ -7904,6 +8551,13 @@
       </x:c>
       <x:c r="T91" s="78"/>
       <x:c r="U91" s="78"/>
+      <x:c r="V91" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W91" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X91" s="78"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="40" t="n">
@@ -7975,10 +8629,17 @@
         <x:v>An empty chair, a canceled plan, or a quiet phone can feel like proof that love has gone missing. You respond by becoming more responsible, less demanding, and harder to reach, which makes the loneliness even less visible. The square turns absence into a strict conclusion. A difficult night is still one night, not the final record of every relationship.</x:v>
       </x:c>
       <x:c r="S92" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T92" s="78"/>
       <x:c r="U92" s="78"/>
+      <x:c r="V92" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W92" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X92" s="78"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="41" t="n">
@@ -8052,6 +8713,13 @@
       </x:c>
       <x:c r="T93" s="78"/>
       <x:c r="U93" s="78"/>
+      <x:c r="V93" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W93" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X93" s="78"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="40" t="n">
@@ -8123,10 +8791,17 @@
         <x:v>A changed reservation or unexpected message can overturn the mood faster than the plan itself requires. You need a different room, a different answer, or immediate space, and everybody else is still trying to understand what changed. The square makes surprise land directly in the feelings. Adaptation gets easier when the first reaction is not treated as the only possible plan.</x:v>
       </x:c>
       <x:c r="S94" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T94" s="78"/>
       <x:c r="U94" s="78"/>
+      <x:c r="V94" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W94" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X94" s="78"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="41" t="n">
@@ -8198,10 +8873,17 @@
         <x:v>You can read a compliment, invitation, or warm reply as proof that the whole relationship is safe. When the message does not come, the mood drops before there is enough information to explain why. Approval and emotional security press against each other here. Affection feels more dependable when it is not asked to settle every doubt at once.</x:v>
       </x:c>
       <x:c r="S95" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T95" s="78"/>
       <x:c r="U95" s="78"/>
+      <x:c r="V95" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W95" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X95" s="78"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="40" t="n">
@@ -8275,6 +8957,13 @@
       </x:c>
       <x:c r="T96" s="78"/>
       <x:c r="U96" s="78"/>
+      <x:c r="V96" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W96" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X96" s="78"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="41" t="n">
@@ -8346,10 +9035,17 @@
         <x:v>You are often able to make a difficult room feel more possible without pretending the problem is small. Food appears, another chair is found, and somebody remembers that the week contains more than the current disappointment. Confidence and feeling support each other naturally here. The ease is generous, though it can also add one more promise to a calendar that was already full.</x:v>
       </x:c>
       <x:c r="S97" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T97" s="78"/>
       <x:c r="U97" s="78"/>
+      <x:c r="V97" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W97" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X97" s="78"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="40" t="n">
@@ -8421,10 +9117,17 @@
         <x:v>When something matters, feeling moves into action without much delay. You make the call, carry the box, defend the friend, or start the repair while other people are still deciding how upset they are. Courage has emotional fuel here, and the body usually knows where to put it. The action is strongest when it serves the feeling instead of turning every feeling into a fight.</x:v>
       </x:c>
       <x:c r="S98" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T98" s="78"/>
       <x:c r="U98" s="78"/>
+      <x:c r="V98" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W98" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X98" s="78"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="41" t="n">
@@ -8496,10 +9199,17 @@
         <x:v>You can usually find the sentence that tells the truth about a feeling without making it larger than it is. A difficult text gets written, a memory is explained clearly, and another person can follow how the reaction connects to what happened. Thought gives emotion a usable shape here. The words tend to help because they carry both the fact and the human consequence.</x:v>
       </x:c>
       <x:c r="S99" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T99" s="78"/>
       <x:c r="U99" s="78"/>
+      <x:c r="V99" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W99" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X99" s="78"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="40" t="n">
@@ -8573,6 +9283,13 @@
       </x:c>
       <x:c r="T100" s="78"/>
       <x:c r="U100" s="78"/>
+      <x:c r="V100" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W100" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X100" s="78"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="41" t="n">
@@ -8644,10 +9361,17 @@
         <x:v>You notice the music that changes the room, the book that gives somebody language for a difficult week, or the quiet job nobody else realized needed doing. Sensitivity moves easily toward images, stories, and acts of service. That can make art and care feel instinctive. It also means the atmosphere enters quickly, so choosing where to spend an evening matters.</x:v>
       </x:c>
       <x:c r="S101" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T101" s="78"/>
       <x:c r="U101" s="78"/>
+      <x:c r="V101" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W101" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X101" s="78"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="40" t="n">
@@ -8721,6 +9445,13 @@
       </x:c>
       <x:c r="T102" s="78"/>
       <x:c r="U102" s="78"/>
+      <x:c r="V102" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W102" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X102" s="78"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="41" t="n">
@@ -8792,10 +9523,17 @@
         <x:v>You can stay in the conversation after another person admits the part they expected to hide. Strong feelings do not automatically send you out of the room, and difficult truths often make the exchange clearer rather than more frightening. Emotional depth and honesty cooperate here. People may tell you more because they sense that the real subject will not be avoided.</x:v>
       </x:c>
       <x:c r="S103" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T103" s="78"/>
       <x:c r="U103" s="78"/>
+      <x:c r="V103" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W103" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X103" s="78"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="40" t="n">
@@ -8867,10 +9605,17 @@
         <x:v>You can keep dinner warm, finish the form, or make the necessary call while the day is emotionally difficult. Feeling does not disappear, but it has enough structure to move beside responsibility. Other people often rely on that steadiness because it does not demand that the room become calm first. The support is quiet, practical, and usually visible in what got done.</x:v>
       </x:c>
       <x:c r="S104" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T104" s="78"/>
       <x:c r="U104" s="78"/>
+      <x:c r="V104" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W104" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X104" s="78"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="41" t="n">
@@ -8944,6 +9689,13 @@
       </x:c>
       <x:c r="T105" s="78"/>
       <x:c r="U105" s="78"/>
+      <x:c r="V105" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W105" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X105" s="78"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="40" t="n">
@@ -9015,10 +9767,17 @@
         <x:v>A changed plan can become a different good evening before anybody has time to mourn the original reservation. You adjust the room, try the new route, or make space for an unexpected person without losing the emotional thread of the day. Feeling and change cooperate easily here. The mood can move without having to declare the first plan a mistake.</x:v>
       </x:c>
       <x:c r="S106" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T106" s="78"/>
       <x:c r="U106" s="78"/>
+      <x:c r="V106" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W106" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X106" s="78"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="41" t="n">
@@ -9090,10 +9849,17 @@
         <x:v>You remember the coffee order, bring food when someone has had a terrible week, and notice when the room would feel better with the lamp on instead of the overhead light. Affection tends to come through small choices that make another person more comfortable. You may not think of any of this as caretaking. To the people who know you well, it is often how they know you care.</x:v>
       </x:c>
       <x:c r="S107" s="69" t="str">
-        <x:v>PASS: mechanism lint + prior-structure comparison</x:v>
+        <x:v>DETERMINISTIC CLEAR ONLY — semantic owner review pending</x:v>
       </x:c>
       <x:c r="T107" s="78"/>
       <x:c r="U107" s="78"/>
+      <x:c r="V107" s="81" t="str">
+        <x:v>CLEAR: at least one observable clause (necessary, not sufficient)</x:v>
+      </x:c>
+      <x:c r="W107" s="81" t="str">
+        <x:v>PENDING OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="X107" s="78"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="40" t="n">
@@ -9167,6 +9933,13 @@
       </x:c>
       <x:c r="T108" s="78"/>
       <x:c r="U108" s="78"/>
+      <x:c r="V108" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W108" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X108" s="78"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="41" t="n">
@@ -9240,6 +10013,13 @@
       </x:c>
       <x:c r="T109" s="78"/>
       <x:c r="U109" s="78"/>
+      <x:c r="V109" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W109" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X109" s="78"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="40" t="n">
@@ -9313,6 +10093,13 @@
       </x:c>
       <x:c r="T110" s="78"/>
       <x:c r="U110" s="78"/>
+      <x:c r="V110" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W110" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X110" s="78"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="41" t="n">
@@ -9386,6 +10173,13 @@
       </x:c>
       <x:c r="T111" s="78"/>
       <x:c r="U111" s="78"/>
+      <x:c r="V111" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W111" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X111" s="78"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="40" t="n">
@@ -9459,6 +10253,13 @@
       </x:c>
       <x:c r="T112" s="78"/>
       <x:c r="U112" s="78"/>
+      <x:c r="V112" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W112" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X112" s="78"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="41" t="n">
@@ -9532,6 +10333,13 @@
       </x:c>
       <x:c r="T113" s="78"/>
       <x:c r="U113" s="78"/>
+      <x:c r="V113" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W113" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X113" s="78"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="40" t="n">
@@ -9605,6 +10413,13 @@
       </x:c>
       <x:c r="T114" s="78"/>
       <x:c r="U114" s="78"/>
+      <x:c r="V114" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W114" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X114" s="78"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="41" t="n">
@@ -9678,6 +10493,13 @@
       </x:c>
       <x:c r="T115" s="78"/>
       <x:c r="U115" s="78"/>
+      <x:c r="V115" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W115" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X115" s="78"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="40" t="n">
@@ -9751,6 +10573,13 @@
       </x:c>
       <x:c r="T116" s="78"/>
       <x:c r="U116" s="78"/>
+      <x:c r="V116" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W116" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X116" s="78"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="41" t="n">
@@ -9824,6 +10653,13 @@
       </x:c>
       <x:c r="T117" s="78"/>
       <x:c r="U117" s="78"/>
+      <x:c r="V117" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W117" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X117" s="78"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="40" t="n">
@@ -9897,6 +10733,13 @@
       </x:c>
       <x:c r="T118" s="78"/>
       <x:c r="U118" s="78"/>
+      <x:c r="V118" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W118" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X118" s="78"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="41" t="n">
@@ -9970,6 +10813,13 @@
       </x:c>
       <x:c r="T119" s="78"/>
       <x:c r="U119" s="78"/>
+      <x:c r="V119" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W119" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X119" s="78"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="40" t="n">
@@ -10043,6 +10893,13 @@
       </x:c>
       <x:c r="T120" s="78"/>
       <x:c r="U120" s="78"/>
+      <x:c r="V120" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W120" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X120" s="78"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="41" t="n">
@@ -10116,6 +10973,13 @@
       </x:c>
       <x:c r="T121" s="78"/>
       <x:c r="U121" s="78"/>
+      <x:c r="V121" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W121" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X121" s="78"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="40" t="n">
@@ -10189,6 +11053,13 @@
       </x:c>
       <x:c r="T122" s="78"/>
       <x:c r="U122" s="78"/>
+      <x:c r="V122" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W122" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X122" s="78"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="41" t="n">
@@ -10262,6 +11133,13 @@
       </x:c>
       <x:c r="T123" s="78"/>
       <x:c r="U123" s="78"/>
+      <x:c r="V123" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W123" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X123" s="78"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="40" t="n">
@@ -10335,6 +11213,13 @@
       </x:c>
       <x:c r="T124" s="78"/>
       <x:c r="U124" s="78"/>
+      <x:c r="V124" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W124" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X124" s="78"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="41" t="n">
@@ -10408,6 +11293,13 @@
       </x:c>
       <x:c r="T125" s="78"/>
       <x:c r="U125" s="78"/>
+      <x:c r="V125" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W125" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X125" s="78"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="40" t="n">
@@ -10481,6 +11373,13 @@
       </x:c>
       <x:c r="T126" s="78"/>
       <x:c r="U126" s="78"/>
+      <x:c r="V126" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W126" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X126" s="78"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="41" t="n">
@@ -10554,6 +11453,13 @@
       </x:c>
       <x:c r="T127" s="78"/>
       <x:c r="U127" s="78"/>
+      <x:c r="V127" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W127" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X127" s="78"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="40" t="n">
@@ -10627,6 +11533,13 @@
       </x:c>
       <x:c r="T128" s="78"/>
       <x:c r="U128" s="78"/>
+      <x:c r="V128" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W128" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X128" s="78"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="41" t="n">
@@ -10700,6 +11613,13 @@
       </x:c>
       <x:c r="T129" s="78"/>
       <x:c r="U129" s="78"/>
+      <x:c r="V129" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W129" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X129" s="78"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="40" t="n">
@@ -10773,6 +11693,13 @@
       </x:c>
       <x:c r="T130" s="78"/>
       <x:c r="U130" s="78"/>
+      <x:c r="V130" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W130" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X130" s="78"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="41" t="n">
@@ -10846,6 +11773,13 @@
       </x:c>
       <x:c r="T131" s="78"/>
       <x:c r="U131" s="78"/>
+      <x:c r="V131" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W131" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X131" s="78"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="40" t="n">
@@ -10919,6 +11853,13 @@
       </x:c>
       <x:c r="T132" s="78"/>
       <x:c r="U132" s="78"/>
+      <x:c r="V132" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W132" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X132" s="78"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="41" t="n">
@@ -10992,6 +11933,13 @@
       </x:c>
       <x:c r="T133" s="78"/>
       <x:c r="U133" s="78"/>
+      <x:c r="V133" s="81" t="str">
+        <x:v>NOT RUN</x:v>
+      </x:c>
+      <x:c r="W133" s="81" t="str">
+        <x:v>SOURCE_GAP</x:v>
+      </x:c>
+      <x:c r="X133" s="78"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -11015,88 +11963,112 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="80" t="str">
+      <x:c r="A1" s="83" t="str">
         <x:v>LL V13 WP-1 Batch 1 — V3 author-from-mechanism review</x:v>
       </x:c>
-      <x:c r="B1" s="80"/>
+      <x:c r="B1" s="83"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="83" t="str">
+      <x:c r="A3" s="86" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="86" t="str">
+      <x:c r="B3" s="89" t="str">
         <x:v>Review-gated editorial candidates only. No row is approved, canonical, served, auto-published, or promoted.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="83" t="str">
+      <x:c r="A4" s="86" t="str">
         <x:v>Writer source</x:v>
       </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="B4" s="89" t="str">
         <x:v>Exact-key AstrologySupport plus source constraints and 4–6 exact_owner_approved passages from at least 3 source rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
-      <x:c r="A5" s="83" t="str">
+      <x:c r="A5" s="86" t="str">
         <x:v>Prior prose</x:v>
       </x:c>
-      <x:c r="B5" s="86" t="str">
+      <x:c r="B5" s="89" t="str">
         <x:v>Excluded from the writer packet by construction. V2/current prose is available only to the downstream structural comparison.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="83" t="str">
+      <x:c r="A6" s="86" t="str">
         <x:v>Coverage</x:v>
       </x:c>
-      <x:c r="B6" s="86" t="str">
+      <x:c r="B6" s="89" t="str">
         <x:v>51 of 132 rows READY; 81 remain SOURCE_GAP and have no V3 copy.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="83" t="str">
+      <x:c r="A7" s="86" t="str">
         <x:v>713-row audit</x:v>
       </x:c>
-      <x:c r="B7" s="86" t="str">
+      <x:c r="B7" s="89" t="str">
         <x:v>266 of 713 compliant today (37.31%); all 713 have AstrologySupport. Remaining rows fail closed on registry boundary or unsupported key shape.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="83" t="str">
-        <x:v>Deterministic gates</x:v>
-      </x:c>
-      <x:c r="B8" s="86" t="str">
-        <x:v>Abstract-noun opening, zero concrete nouns, therapy-register cluster without observable action, photograph test, trait entry, archetype soup, and paraphrase of prior.</x:v>
+      <x:c r="A8" s="86" t="str">
+        <x:v>Deterministic precheck</x:v>
+      </x:c>
+      <x:c r="B8" s="89" t="str">
+        <x:v>Abstract-noun opening, zero concrete nouns, therapy-register cluster without observable action, photograph minimum, trait entry, known astrology-summary patterns, archetype soup, and paraphrase of prior. A clear result is not an editorial verdict.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="83" t="str">
+      <x:c r="A9" s="86" t="str">
+        <x:v>Photograph rule</x:v>
+      </x:c>
+      <x:c r="B9" s="89" t="str">
+        <x:v>A passage does not pass because it contains one photographable clause. Every sentence must advance the lived scene, state a specific consequence, or provide necessary astrology-to-life perspective.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="86" t="str">
+        <x:v>Metric limit</x:v>
+      </x:c>
+      <x:c r="B10" s="89" t="str">
+        <x:v>Observable-noun density is lint only. It does not prove voice quality, coherent causal scene density, or that one model's batch is better.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="86" t="str">
         <x:v>Semantic owner gate</x:v>
       </x:c>
-      <x:c r="B9" s="86" t="str">
-        <x:v>Photograph-test, trait-entry, interchangeable, astrology-summary, archetype-soup, and paraphrase-of-prior remain blocking owner-review checks.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="83" t="str">
+      <x:c r="B11" s="89" t="str">
+        <x:v>Review each READY row as prose. Trait-entry, interchangeable, astrology-summary, archetype-soup, paraphrase-of-prior, and whole-passage sentence role remain blocking owner-review checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="86" t="str">
+        <x:v>Evidence boundary</x:v>
+      </x:c>
+      <x:c r="B12" s="89" t="str">
+        <x:v>Exactly 81 rows involve Ascendant, Midheaven, North Node, South Node, or Part of Fortune. Those are exactly the 81 SOURCE_GAP rows; all 51 non-point rows are READY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="86" t="str">
         <x:v>Owner action</x:v>
       </x:c>
-      <x:c r="B10" s="86" t="str">
+      <x:c r="B13" s="89" t="str">
         <x:v>Review only rows marked READY. Enter approve/edit/cut in V3 owner verdict; an edit requires exact final wording in V3 owner edit. SOURCE_GAP rows remain blank.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="83" t="str">
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="86" t="str">
         <x:v>V2 preservation</x:v>
       </x:c>
-      <x:c r="B11" s="86" t="str">
-        <x:v>Candidates132 columns A:O are imported from V2 without intentional cell changes. V3 evidence occupies P:U.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="83" t="str">
+      <x:c r="B14" s="89" t="str">
+        <x:v>Candidates132 columns A:O are imported from V2 without intentional cell changes. V3 evidence occupies P:X.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="86" t="str">
         <x:v>Batches</x:v>
       </x:c>
-      <x:c r="B12" s="86" t="str">
+      <x:c r="B15" s="89" t="str">
         <x:v>Batches 3 through 6 remain unstarted.</x:v>
       </x:c>
     </x:row>

</xml_diff>